<commit_message>
Test plan BRD-1 New Business; builder sorts BRD IDs and halves long tables
brd01_cases.yaml covers the 93 FRs of FRS BRD-1 with 237 conditions and 386
cases, 311 of them tied to existing automated tests, plus the roles-and-access
checks and seven FRS findings. The builder now drops page notes from BRD
references, sorts BRD IDs by number and sets long coverage tables side by
side so the Word summary stays within 20 pages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/TestPlans/BIBS_TestPlan_BRD-03_Product_Maintenance_v1.0.xlsx
+++ b/docs/deliverables/out/TestPlans/BIBS_TestPlan_BRD-03_Product_Maintenance_v1.0.xlsx
@@ -1330,12 +1330,12 @@
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>The FRS gives the log-in and lock-out messages without codes and the threshold only as "configured". The build locks at 5 failed attempts by default and the log-in endpoint also rate-limits (LOGIN_RATE_LIMITED, HTTP 429), which the FRS does not mention.</t>
+          <t>The FRS messages "Invalid user ID or password" and "Your account is locked. Contact the System Administrator" differ from the build ("Invalid user name or password", "Account is locked. Contact your administrator.", code AUTHENTICATION_FAILED). The threshold is given only as "configured"; the build reads LOGIN_MAX_FAILED_ATTEMPTS (3 as delivered). The log-in endpoint also rate-limits (LOGIN_RATE_LIMITED, HTTP 429), which the FRS does not mention.</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Name the parameter and default of the lock-out threshold and add the rate limit to FR-PM-001.</t>
+          <t>Quote the built messages and code, name the parameter and its value, and add the rate limit to FR-PM-001.</t>
         </is>
       </c>
     </row>
@@ -8203,7 +8203,7 @@
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>Parameter of the session policy shows the lock-out threshold (default 5).
+          <t>Administration &gt; System Parameters shows LOGIN_MAX_FAILED_ATTEMPTS (3 as delivered).
 Data: TD-PM-01 Demo users and roles</t>
         </is>
       </c>
@@ -26458,7 +26458,7 @@
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>PMADD05</t>
+          <t>BRPM.003</t>
         </is>
       </c>
       <c r="B46" s="12" t="inlineStr">
@@ -26469,23 +26469,23 @@
       <c r="C46" s="12" t="inlineStr"/>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-002, FR-PM-003</t>
+          <t>FR-PM-012</t>
         </is>
       </c>
       <c r="E46" s="12" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F46" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G46" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="G46" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="H46" s="12" t="n">
-        <v>12</v>
-      </c>
       <c r="I46" s="12" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J46" s="27" t="inlineStr">
         <is>
@@ -26496,7 +26496,7 @@
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>BRPM.020</t>
+          <t>BRPM.004</t>
         </is>
       </c>
       <c r="B47" s="12" t="inlineStr">
@@ -26507,20 +26507,20 @@
       <c r="C47" s="12" t="inlineStr"/>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-004</t>
+          <t>FR-PM-012</t>
         </is>
       </c>
       <c r="E47" s="12" t="n">
         <v>3</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G47" s="12" t="n">
         <v>2</v>
       </c>
       <c r="H47" s="12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I47" s="12" t="n">
         <v>3</v>
@@ -26534,7 +26534,7 @@
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t>BRPM.024</t>
+          <t>BRPM.005</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
@@ -26545,7 +26545,7 @@
       <c r="C48" s="12" t="inlineStr"/>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-005</t>
+          <t>FR-PM-013</t>
         </is>
       </c>
       <c r="E48" s="12" t="n">
@@ -26572,7 +26572,7 @@
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t>PMADD01</t>
+          <t>BRPM.006</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -26583,23 +26583,23 @@
       <c r="C49" s="12" t="inlineStr"/>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-010</t>
+          <t>FR-PM-045, FR-PM-052, FR-PM-071</t>
         </is>
       </c>
       <c r="E49" s="12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G49" s="12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H49" s="12" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="I49" s="12" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J49" s="27" t="inlineStr">
         <is>
@@ -26610,7 +26610,7 @@
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t>PMADD02</t>
+          <t>BRPM.007</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
@@ -26621,23 +26621,23 @@
       <c r="C50" s="12" t="inlineStr"/>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-011, FR-PM-014</t>
+          <t>FR-PM-050, FR-PM-051</t>
         </is>
       </c>
       <c r="E50" s="12" t="n">
         <v>7</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G50" s="12" t="n">
         <v>6</v>
       </c>
       <c r="H50" s="12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I50" s="12" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J50" s="27" t="inlineStr">
         <is>
@@ -26648,7 +26648,7 @@
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>BRPM.003</t>
+          <t>BRPM.008</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -26659,23 +26659,23 @@
       <c r="C51" s="12" t="inlineStr"/>
       <c r="D51" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-012</t>
+          <t>FR-PM-020, FR-PM-021</t>
         </is>
       </c>
       <c r="E51" s="12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G51" s="12" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H51" s="12" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="I51" s="12" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J51" s="27" t="inlineStr">
         <is>
@@ -26686,7 +26686,7 @@
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>BRPM.004</t>
+          <t>BRPM.009</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
@@ -26697,23 +26697,23 @@
       <c r="C52" s="12" t="inlineStr"/>
       <c r="D52" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-012</t>
+          <t>FR-PM-022, FR-PM-023</t>
         </is>
       </c>
       <c r="E52" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="F52" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="G52" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="F52" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G52" s="12" t="n">
-        <v>2</v>
-      </c>
       <c r="H52" s="12" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I52" s="12" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J52" s="27" t="inlineStr">
         <is>
@@ -26724,7 +26724,7 @@
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>BRPM.005</t>
+          <t>BRPM.010</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -26735,23 +26735,23 @@
       <c r="C53" s="12" t="inlineStr"/>
       <c r="D53" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-013</t>
+          <t>FR-PM-032, FR-PM-033, FR-PM-036</t>
         </is>
       </c>
       <c r="E53" s="12" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F53" s="12" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G53" s="12" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H53" s="12" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="I53" s="12" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J53" s="27" t="inlineStr">
         <is>
@@ -26762,7 +26762,7 @@
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>BRPM.008</t>
+          <t>BRPM.011</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
@@ -26773,23 +26773,23 @@
       <c r="C54" s="12" t="inlineStr"/>
       <c r="D54" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-020, FR-PM-021</t>
+          <t>FR-PM-020, FR-PM-024, FR-PM-045</t>
         </is>
       </c>
       <c r="E54" s="12" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F54" s="12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G54" s="12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H54" s="12" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I54" s="12" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J54" s="27" t="inlineStr">
         <is>
@@ -26800,7 +26800,7 @@
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>BRPM.011</t>
+          <t>BRPM.012</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -26811,23 +26811,23 @@
       <c r="C55" s="12" t="inlineStr"/>
       <c r="D55" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-020, FR-PM-024, FR-PM-045</t>
+          <t>FR-PM-030</t>
         </is>
       </c>
       <c r="E55" s="12" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F55" s="12" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G55" s="12" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H55" s="12" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="I55" s="12" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="J55" s="27" t="inlineStr">
         <is>
@@ -26838,7 +26838,7 @@
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
         <is>
-          <t>BRPM.021</t>
+          <t>BRPM.013</t>
         </is>
       </c>
       <c r="B56" s="12" t="inlineStr">
@@ -26849,23 +26849,23 @@
       <c r="C56" s="12" t="inlineStr"/>
       <c r="D56" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-021, FR-PM-073</t>
+          <t>FR-PM-031, FR-PM-034, FR-PM-036</t>
         </is>
       </c>
       <c r="E56" s="12" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G56" s="12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H56" s="12" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="I56" s="12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J56" s="27" t="inlineStr">
         <is>
@@ -26876,7 +26876,7 @@
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>BRPM.009</t>
+          <t>BRPM.014</t>
         </is>
       </c>
       <c r="B57" s="12" t="inlineStr">
@@ -26887,23 +26887,23 @@
       <c r="C57" s="12" t="inlineStr"/>
       <c r="D57" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-022, FR-PM-023</t>
+          <t>FR-PM-034</t>
         </is>
       </c>
       <c r="E57" s="12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G57" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H57" s="12" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I57" s="12" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J57" s="27" t="inlineStr">
         <is>
@@ -26914,7 +26914,7 @@
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
         <is>
-          <t>BRPM.012</t>
+          <t>BRPM.015</t>
         </is>
       </c>
       <c r="B58" s="12" t="inlineStr">
@@ -26925,23 +26925,23 @@
       <c r="C58" s="12" t="inlineStr"/>
       <c r="D58" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-030</t>
+          <t>FR-PM-040, FR-PM-041, FR-PM-042, FR-PM-043</t>
         </is>
       </c>
       <c r="E58" s="12" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G58" s="12" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H58" s="12" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="I58" s="12" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="J58" s="27" t="inlineStr">
         <is>
@@ -26952,7 +26952,7 @@
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>BRPM.013</t>
+          <t>BRPM.016</t>
         </is>
       </c>
       <c r="B59" s="12" t="inlineStr">
@@ -26963,23 +26963,23 @@
       <c r="C59" s="12" t="inlineStr"/>
       <c r="D59" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-031, FR-PM-034, FR-PM-036</t>
+          <t>FR-PM-044</t>
         </is>
       </c>
       <c r="E59" s="12" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G59" s="12" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H59" s="12" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="I59" s="12" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="J59" s="27" t="inlineStr">
         <is>
@@ -26990,7 +26990,7 @@
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t>PMADD04</t>
+          <t>BRPM.017</t>
         </is>
       </c>
       <c r="B60" s="12" t="inlineStr">
@@ -27001,23 +27001,23 @@
       <c r="C60" s="12" t="inlineStr"/>
       <c r="D60" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-031, FR-PM-032</t>
+          <t>FR-PM-044, FR-PM-060, FR-PM-061, FR-PM-071</t>
         </is>
       </c>
       <c r="E60" s="12" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G60" s="12" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H60" s="12" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="I60" s="12" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="J60" s="27" t="inlineStr">
         <is>
@@ -27028,7 +27028,7 @@
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t>BRPM.010</t>
+          <t>BRPM.018</t>
         </is>
       </c>
       <c r="B61" s="12" t="inlineStr">
@@ -27039,23 +27039,23 @@
       <c r="C61" s="12" t="inlineStr"/>
       <c r="D61" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-032, FR-PM-033, FR-PM-036</t>
+          <t>FR-PM-071</t>
         </is>
       </c>
       <c r="E61" s="12" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G61" s="12" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H61" s="12" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="I61" s="12" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J61" s="27" t="inlineStr">
         <is>
@@ -27066,7 +27066,7 @@
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
         <is>
-          <t>BRPM.014</t>
+          <t>BRPM.019</t>
         </is>
       </c>
       <c r="B62" s="12" t="inlineStr">
@@ -27077,11 +27077,11 @@
       <c r="C62" s="12" t="inlineStr"/>
       <c r="D62" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-034</t>
+          <t>FR-PM-070</t>
         </is>
       </c>
       <c r="E62" s="12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F62" s="12" t="n">
         <v>3</v>
@@ -27093,7 +27093,7 @@
         <v>5</v>
       </c>
       <c r="I62" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J62" s="27" t="inlineStr">
         <is>
@@ -27104,7 +27104,7 @@
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
         <is>
-          <t>PMADD03</t>
+          <t>BRPM.020</t>
         </is>
       </c>
       <c r="B63" s="12" t="inlineStr">
@@ -27115,7 +27115,7 @@
       <c r="C63" s="12" t="inlineStr"/>
       <c r="D63" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-035</t>
+          <t>FR-PM-004</t>
         </is>
       </c>
       <c r="E63" s="12" t="n">
@@ -27125,13 +27125,13 @@
         <v>2</v>
       </c>
       <c r="G63" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H63" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="I63" s="12" t="n">
         <v>3</v>
-      </c>
-      <c r="H63" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="I63" s="12" t="n">
-        <v>2</v>
       </c>
       <c r="J63" s="27" t="inlineStr">
         <is>
@@ -27142,7 +27142,7 @@
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
         <is>
-          <t>BRPM.015</t>
+          <t>BRPM.021</t>
         </is>
       </c>
       <c r="B64" s="12" t="inlineStr">
@@ -27153,23 +27153,23 @@
       <c r="C64" s="12" t="inlineStr"/>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-040, FR-PM-041, FR-PM-042, FR-PM-043</t>
+          <t>FR-PM-021, FR-PM-073</t>
         </is>
       </c>
       <c r="E64" s="12" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F64" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="G64" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="H64" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="G64" s="12" t="n">
-        <v>17</v>
-      </c>
-      <c r="H64" s="12" t="n">
-        <v>27</v>
-      </c>
       <c r="I64" s="12" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="J64" s="27" t="inlineStr">
         <is>
@@ -27180,7 +27180,7 @@
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
         <is>
-          <t>PMADD06</t>
+          <t>BRPM.022</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -27191,23 +27191,23 @@
       <c r="C65" s="12" t="inlineStr"/>
       <c r="D65" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-043</t>
+          <t>FR-PM-072</t>
         </is>
       </c>
       <c r="E65" s="12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F65" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G65" s="12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H65" s="12" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I65" s="12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J65" s="27" t="inlineStr">
         <is>
@@ -27218,7 +27218,7 @@
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
         <is>
-          <t>BRPM.016</t>
+          <t>BRPM.024</t>
         </is>
       </c>
       <c r="B66" s="12" t="inlineStr">
@@ -27229,23 +27229,23 @@
       <c r="C66" s="12" t="inlineStr"/>
       <c r="D66" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-044</t>
+          <t>FR-PM-005</t>
         </is>
       </c>
       <c r="E66" s="12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F66" s="12" t="n">
         <v>2</v>
       </c>
       <c r="G66" s="12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H66" s="12" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I66" s="12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J66" s="27" t="inlineStr">
         <is>
@@ -27256,7 +27256,7 @@
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
         <is>
-          <t>BRPM.017</t>
+          <t>PMADD01</t>
         </is>
       </c>
       <c r="B67" s="12" t="inlineStr">
@@ -27267,23 +27267,23 @@
       <c r="C67" s="12" t="inlineStr"/>
       <c r="D67" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-044, FR-PM-060, FR-PM-061, FR-PM-071</t>
+          <t>FR-PM-010</t>
         </is>
       </c>
       <c r="E67" s="12" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="F67" s="12" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="G67" s="12" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H67" s="12" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="J67" s="27" t="inlineStr">
         <is>
@@ -27294,7 +27294,7 @@
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
         <is>
-          <t>BRPM.006</t>
+          <t>PMADD02</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
@@ -27305,23 +27305,23 @@
       <c r="C68" s="12" t="inlineStr"/>
       <c r="D68" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-045, FR-PM-052, FR-PM-071</t>
+          <t>FR-PM-011, FR-PM-014</t>
         </is>
       </c>
       <c r="E68" s="12" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F68" s="12" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G68" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H68" s="12" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I68" s="12" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J68" s="27" t="inlineStr">
         <is>
@@ -27332,7 +27332,7 @@
     <row r="69">
       <c r="A69" s="12" t="inlineStr">
         <is>
-          <t>BRPM.007</t>
+          <t>PMADD03</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
@@ -27343,23 +27343,23 @@
       <c r="C69" s="12" t="inlineStr"/>
       <c r="D69" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-050, FR-PM-051</t>
+          <t>FR-PM-035</t>
         </is>
       </c>
       <c r="E69" s="12" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G69" s="12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H69" s="12" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I69" s="12" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J69" s="27" t="inlineStr">
         <is>
@@ -27370,7 +27370,7 @@
     <row r="70">
       <c r="A70" s="12" t="inlineStr">
         <is>
-          <t>BRPM.019</t>
+          <t>PMADD04</t>
         </is>
       </c>
       <c r="B70" s="12" t="inlineStr">
@@ -27381,23 +27381,23 @@
       <c r="C70" s="12" t="inlineStr"/>
       <c r="D70" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-070</t>
+          <t>FR-PM-031, FR-PM-032</t>
         </is>
       </c>
       <c r="E70" s="12" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G70" s="12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H70" s="12" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I70" s="12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J70" s="27" t="inlineStr">
         <is>
@@ -27408,7 +27408,7 @@
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t>BRPM.018</t>
+          <t>PMADD05</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -27419,23 +27419,23 @@
       <c r="C71" s="12" t="inlineStr"/>
       <c r="D71" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-071</t>
+          <t>FR-PM-002, FR-PM-003</t>
         </is>
       </c>
       <c r="E71" s="12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G71" s="12" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H71" s="12" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I71" s="12" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J71" s="27" t="inlineStr">
         <is>
@@ -27446,7 +27446,7 @@
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
         <is>
-          <t>BRPM.022</t>
+          <t>PMADD06</t>
         </is>
       </c>
       <c r="B72" s="12" t="inlineStr">
@@ -27457,23 +27457,23 @@
       <c r="C72" s="12" t="inlineStr"/>
       <c r="D72" s="12" t="inlineStr">
         <is>
-          <t>FR-PM-072</t>
+          <t>FR-PM-043</t>
         </is>
       </c>
       <c r="E72" s="12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F72" s="12" t="n">
         <v>3</v>
       </c>
       <c r="G72" s="12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H72" s="12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I72" s="12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J72" s="27" t="inlineStr">
         <is>

</xml_diff>